<commit_message>
Update task_breakdown with latest numbers
</commit_message>
<xml_diff>
--- a/data/task_breakdown.xlsx
+++ b/data/task_breakdown.xlsx
@@ -511,8 +511,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D9F28F5819300A43901E9DBC513AE4A8" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0baf57f2338ee7e444e82289da7848b2">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40111ba8-f904-4ecf-a49d-62383d8f24ce" xmlns:ns3="1f46f138-9cbd-41b8-9ede-c2ff327f64b5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="02446be83e1a77402352026bad75407b" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D9F28F5819300A43901E9DBC513AE4A8" ma:contentTypeVersion="6" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="25cf4ea28c43452cb8a3259f612469bf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40111ba8-f904-4ecf-a49d-62383d8f24ce" xmlns:ns3="1f46f138-9cbd-41b8-9ede-c2ff327f64b5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a4c398a66158f28d13f94d1796e970fb" ns2:_="" ns3:_="">
     <xsd:import namespace="40111ba8-f904-4ecf-a49d-62383d8f24ce"/>
     <xsd:import namespace="1f46f138-9cbd-41b8-9ede-c2ff327f64b5"/>
     <xsd:element name="properties">
@@ -561,7 +561,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1f46f138-9cbd-41b8-9ede-c2ff327f64b5" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Delt med" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -580,7 +580,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Delt med detaljer" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -597,8 +597,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Indholdstype"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titel"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -705,20 +705,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EC0A359-2A59-4DE4-B71A-F490E89AB2F0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="40111ba8-f904-4ecf-a49d-62383d8f24ce"/>
-    <ds:schemaRef ds:uri="1f46f138-9cbd-41b8-9ede-c2ff327f64b5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53C94D47-C5BB-4265-BCC4-E8B1DF9388A9}"/>
 </file>
</xml_diff>